<commit_message>
Actualización automática: 2026-04-12 17:31
</commit_message>
<xml_diff>
--- a/Fact_Futmondo_2025_26.xlsx
+++ b/Fact_Futmondo_2025_26.xlsx
@@ -5498,7 +5498,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>5f452f5e66dd374930eb2b71</t>
+          <t>62d5bd9ad8106d3355b5bdc1</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -5510,16 +5510,16 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>81.40000000000001</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="E242" t="n">
-        <v>2193.5</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>5f47ab5b9e2edb0bb831c703</t>
+          <t>5f452f5e66dd374930eb2b71</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -5531,16 +5531,16 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>59.5</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="E243" t="n">
-        <v>1746</v>
+        <v>2193.5</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>62d5bd9ad8106d3355b5bdc1</t>
+          <t>5f47ab5b9e2edb0bb831c703</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -5552,16 +5552,16 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>52.6</v>
+        <v>59.5</v>
       </c>
       <c r="E244" t="n">
-        <v>2141.5</v>
+        <v>1746</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>5f4530beec331549297ee6d6</t>
+          <t>5f47aeb6c387a50bca03dd55</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -5573,16 +5573,16 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>46.9</v>
+        <v>52.9</v>
       </c>
       <c r="E245" t="n">
-        <v>2058.2</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>5f47aeb6c387a50bca03dd55</t>
+          <t>5f4530beec331549297ee6d6</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -5594,10 +5594,10 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>42.2</v>
+        <v>48.3</v>
       </c>
       <c r="E246" t="n">
-        <v>1993.3</v>
+        <v>2059.6</v>
       </c>
     </row>
     <row r="247">
@@ -5657,10 +5657,10 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>12.2</v>
+        <v>24.8</v>
       </c>
       <c r="E249" t="n">
-        <v>2082.4</v>
+        <v>2095</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática: 2026-04-16 16:57
</commit_message>
<xml_diff>
--- a/Fact_Futmondo_2025_26.xlsx
+++ b/Fact_Futmondo_2025_26.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,27 +429,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ID_Futmondo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Jornada</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Temporada</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Puntos</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Puntos_Acumulados</t>
         </is>
@@ -5486,7 +5498,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>62d5bd9ad8106d3355b5bdc1</t>
+          <t>5f452f5e66dd374930eb2b71</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -5498,16 +5510,16 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>87.09999999999999</v>
+        <v>100.6</v>
       </c>
       <c r="E242" t="n">
-        <v>2176</v>
+        <v>2212.7</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>5f452f5e66dd374930eb2b71</t>
+          <t>62d5bd9ad8106d3355b5bdc1</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -5519,10 +5531,10 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>81.40000000000001</v>
+        <v>88</v>
       </c>
       <c r="E243" t="n">
-        <v>2193.5</v>
+        <v>2176.9</v>
       </c>
     </row>
     <row r="244">
@@ -5540,16 +5552,16 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>59.5</v>
+        <v>73.7</v>
       </c>
       <c r="E244" t="n">
-        <v>1746</v>
+        <v>1760.2</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>5f47aeb6c387a50bca03dd55</t>
+          <t>5f4530beec331549297ee6d6</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -5561,16 +5573,16 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>52.9</v>
+        <v>70.8</v>
       </c>
       <c r="E245" t="n">
-        <v>2004</v>
+        <v>2082.1</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>5f4530beec331549297ee6d6</t>
+          <t>5f453062ec331549297ee6b8</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -5582,10 +5594,10 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>48.3</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="E246" t="n">
-        <v>2059.6</v>
+        <v>2136.1</v>
       </c>
     </row>
     <row r="247">
@@ -5603,10 +5615,10 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>39.7</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="E247" t="n">
-        <v>2189.7</v>
+        <v>2214.6</v>
       </c>
     </row>
     <row r="248">
@@ -5624,16 +5636,16 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>28.1</v>
+        <v>60.5</v>
       </c>
       <c r="E248" t="n">
-        <v>1862.3</v>
+        <v>1894.7</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>5f453062ec331549297ee6b8</t>
+          <t>5f47aeb6c387a50bca03dd55</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -5645,10 +5657,10 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>24.8</v>
+        <v>55.2</v>
       </c>
       <c r="E249" t="n">
-        <v>2095</v>
+        <v>2006.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>